<commit_message>
Use exact questionnaire field names; add dropdown validation for all multiple-choice fields; add blank template
Co-authored-by: MartinaIjaz <MartinaIjaz@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/questionnaire_output.xlsx
+++ b/questionnaire_output.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Прашалник" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Легенда" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Questionnaire" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Legend" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -148,7 +148,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -543,44 +543,44 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="35" customWidth="1" min="11" max="11"/>
     <col width="27" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
     <col width="24" customWidth="1" min="14" max="14"/>
     <col width="26" customWidth="1" min="15" max="15"/>
-    <col width="35" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="38" customWidth="1" min="16" max="16"/>
+    <col width="38" customWidth="1" min="17" max="17"/>
     <col width="30" customWidth="1" min="18" max="18"/>
-    <col width="32" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
-    <col width="35" customWidth="1" min="21" max="21"/>
+    <col width="33" customWidth="1" min="19" max="19"/>
+    <col width="38" customWidth="1" min="20" max="20"/>
+    <col width="38" customWidth="1" min="21" max="21"/>
     <col width="26" customWidth="1" min="22" max="22"/>
-    <col width="27" customWidth="1" min="23" max="23"/>
-    <col width="35" customWidth="1" min="24" max="24"/>
-    <col width="34" customWidth="1" min="25" max="25"/>
-    <col width="35" customWidth="1" min="26" max="26"/>
-    <col width="35" customWidth="1" min="27" max="27"/>
-    <col width="34" customWidth="1" min="28" max="28"/>
+    <col width="38" customWidth="1" min="23" max="23"/>
+    <col width="38" customWidth="1" min="24" max="24"/>
+    <col width="38" customWidth="1" min="25" max="25"/>
+    <col width="38" customWidth="1" min="26" max="26"/>
+    <col width="38" customWidth="1" min="27" max="27"/>
+    <col width="38" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1">
+    <row r="1" ht="50" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REDI Staff Member Name</t>
+          <t>REDI staff member name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Date of Mapping</t>
+          <t>Date of mapping (today)</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Contact Phone Number</t>
+          <t>Contact Phone number</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Place of Residence (Municipality / City)</t>
+          <t>Place of Residence (Municipality, City)</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>Year of Birth</t>
+          <t>Year of your birth</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>Level of Education</t>
+          <t>What is your level of education?</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="M1" s="2" t="inlineStr">
         <is>
-          <t>If NO Roma – Connection to Roma Community</t>
+          <t>If NO, what is the connection to the Roma community?</t>
         </is>
       </c>
       <c r="N1" s="3" t="inlineStr">
         <is>
-          <t>Business Name</t>
+          <t>Business Name?</t>
         </is>
       </c>
       <c r="O1" s="3" t="inlineStr">
@@ -650,32 +650,32 @@
       </c>
       <c r="P1" s="3" t="inlineStr">
         <is>
-          <t>Short Description of the Business</t>
+          <t>Short description of the business. What is your business about?</t>
         </is>
       </c>
       <c r="Q1" s="3" t="inlineStr">
         <is>
-          <t>Business Sector</t>
+          <t>Which business sector does the business belong too?</t>
         </is>
       </c>
       <c r="R1" s="3" t="inlineStr">
         <is>
-          <t>Is the Business Registered?</t>
+          <t>Is the business registered?</t>
         </is>
       </c>
       <c r="S1" s="3" t="inlineStr">
         <is>
-          <t>Date of Business Registration</t>
+          <t>Date of Business Registration?</t>
         </is>
       </c>
       <c r="T1" s="3" t="inlineStr">
         <is>
-          <t>Number of Employees</t>
+          <t>Number of Employees (formal and informal aggregate)</t>
         </is>
       </c>
       <c r="U1" s="3" t="inlineStr">
         <is>
-          <t>Was Business Supported in Phase I?</t>
+          <t>Was your business supported in the Phase I?</t>
         </is>
       </c>
       <c r="V1" s="3" t="inlineStr">
@@ -685,32 +685,32 @@
       </c>
       <c r="W1" s="3" t="inlineStr">
         <is>
-          <t>Type of Service Needed</t>
+          <t>Which type of service do you need? (question for entrepreneurs)</t>
         </is>
       </c>
       <c r="X1" s="3" t="inlineStr">
         <is>
-          <t>Interested in Business Club Membership?</t>
+          <t>Are you interested in a Business Club Membership?</t>
         </is>
       </c>
       <c r="Y1" s="3" t="inlineStr">
         <is>
-          <t>Previously had a Business Loan?</t>
+          <t>Did you previously have a business loan?</t>
         </is>
       </c>
       <c r="Z1" s="3" t="inlineStr">
         <is>
-          <t>Informed about Measures / Help for Business</t>
+          <t>Informed about measure, or anything that helps his business</t>
         </is>
       </c>
       <c r="AA1" s="4" t="inlineStr">
         <is>
-          <t>[REDI Staff] Assessment of Client Needs</t>
+          <t>[For REDI Staff] Describe your assessment of the clients needs</t>
         </is>
       </c>
       <c r="AB1" s="4" t="inlineStr">
         <is>
-          <t>[REDI Staff] Action Recommended</t>
+          <t>[For REDI Staff] Action recommended?</t>
         </is>
       </c>
     </row>
@@ -1543,6 +1543,44 @@
       <c r="AB8" s="8" t="inlineStr"/>
     </row>
   </sheetData>
+  <dataValidations count="12">
+    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Male,Female,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No formal education,Elementary School,High School,University Student,Bachelor,Master,PhD,Vocational Training"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q2:Q500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Agriculture and animal husbandry,Construction,Services (Accounting, Law),Tourism and Hospitality,Beauty and Health,Transportation,Production,Trade,Craftsmanship,Recycling &amp; Upcycling,Cleaning Agency,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="R2:R500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"2020,2021,2022,2023,2024,2025,2026,2027"</formula1>
+    </dataValidation>
+    <dataValidation sqref="W2:W500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Incubation Program,Acceleration Program,Growth Program,Digitalization of the business,One-on-one Mentorship,Business Registration,Brand Identity,Business Plan Writing,Marketing and Promotion,Networking"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X2:X500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No,Maybe"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y2:Y500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z2:Z500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB2:AB500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Develop a business plan,Link to a financial institution (MFI or Bank),Apply for REDI Grant Scheme Support,Link to the Agency of Employment to find or subsidized employment,Link to Government measures, to be self-employed,Train on Business Growth and Development,Business Formalization (Registration),One-on-One Expert Support,Digitalization (Roma Digital Boost),Marketing and Promotion"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1556,67 +1594,67 @@
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>Боја</t>
+          <t>Color Group</t>
         </is>
       </c>
       <c r="B1" s="10" t="inlineStr">
         <is>
-          <t>Значење</t>
+          <t>Fields</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Темно сино / светло сино</t>
+          <t>Dark Blue / Light Blue</t>
         </is>
       </c>
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>Мета-информации (REDI Staff, Датум)</t>
+          <t>REDI Staff Name, Date of Mapping</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1">
+    <row r="3" ht="22" customHeight="1">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>Темно зелено / светло зелено</t>
+          <t>Dark Green / Light Green</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>Лични податоци на клиентот</t>
+          <t>Personal data: Name, Email, Phone, Country, Address, Gender, Education, Roma...</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
+    <row r="4" ht="22" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>Темно кафеаво / светло праскова</t>
+          <t>Dark Brown / Light Peach</t>
         </is>
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>Податоци за бизнис</t>
+          <t>Business data: Business Name, Sector, Registration, Employees, Services...</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
-          <t>Виолетова / светло виолетова</t>
+          <t>Purple / Light Purple</t>
         </is>
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>Проценка и препорака на REDI Staff</t>
+          <t>[For REDI Staff] Assessment &amp; Action Recommended</t>
         </is>
       </c>
     </row>

</xml_diff>